<commit_message>
Add 25 new companies 2026-07-13
</commit_message>
<xml_diff>
--- a/master_companies.xlsx
+++ b/master_companies.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1603,10 +1603,8 @@
           <t>https://dkl-group.co.il/%D7%97%D7%91%D7%A8%D7%AA-%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%91%D7%A0%D7%99%D7%99%D7%A0%D7%99%D7%9D-%D7%A7%D7%98%D7%A0%D7%99%D7%9D/</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>03070308</t>
-        </is>
+      <c r="F36" t="n">
+        <v>3070308</v>
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
@@ -1634,14 +1632,695 @@
           <t>https://www.lior-holdings.co.il/</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>035333372</t>
-        </is>
+      <c r="F37" t="n">
+        <v>35333372</v>
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>ניהול נכסים ודירות בירושלים | חברת ניהול נכסים בי-ם - ברכת הבית</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>ירושלים</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>bhomeisr@gmail.com</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>https://www.bhomeisr.co.il/%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%A0%D7%9B%D7%A1%D7%99%D7%9D-%D7%91%D7%99%D7%A8%D7%95%D7%A9%D7%9C%D7%99%D7%9D/</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>0260601</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr"/>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>קבוצת נתון</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>limort@natoon-group.co.il</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>https://www.natoon-group.co.il/</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>0946182035</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr"/>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>חברת ניהול ואחזקה בעפולה</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>office@paxnihul.co.il</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>https://www.paxnihul.co.il/</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>0547755722</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr"/>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>BEL – אחזקות מבני מגורים, משרדים וקומפלקסים. – BEL מפעילה ...</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>חיפה</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>oshri.biton@gmail.com</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>https://belms.co.il/</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>0547654078</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr"/>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>החברה הכלכלית לקריית גת: עמוד הבית</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>meital@kgat.co.il</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>https://kgat.co.il/</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>0260209</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr"/>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>י.ש.גת</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>office@ysgat.co.il</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>https://www.ysgat.co.il/</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>0230420</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>אום אל-פחם</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>liat.z@enosh.org.il</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>https://www.enosh.org.il/%D7%9E%D7%A8%D7%9B%D7%96%D7%99%D7%9D/%D7%90%D7%95%D7%9D-%D7%90%D7%9C-%D7%A4%D7%97%D7%9D/</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>0250609</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr"/>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>דרופשיפינג - אום אל פחם | הסוכנות לעסקים קטנים</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>mapatz@moital.gov.il</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>https://www.sba.org.il/hb/MaofServices/courses/Pages/Um_El_Fahem/gen-27-10-21.aspx</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>0771233176</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr"/>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>חברת ניהול ואחזקת מבנים ובנייני מגורים / ועד בית | ניהול נכסים פרטיים ...</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>contact@icomplex.co.il</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>https://icomplex.co.il/</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>0777060504</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr"/>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>דף הבית - א-ת ניהול ואחזקת מבנים</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>office@all-service.co.il</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>https://www.all-service.co.il/</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>0220222</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>אחזקת מבנים במעלה אדומים</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>info@calliber.co.il</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>https://calliber.co.il/building-maintenance-maale-adumim/</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>043417951853</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>מעלה אדומים</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>inbalda@mam.org.il</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>https://www.tarbut-hadiur.gov.il/content/142</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>0733485610</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>ניקיון בניינים במעלה אדומים</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>callibenatar@gmail.com</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>https://perfecto-holdings.co.il/building-cleaning-maale-adumim/</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>0250120</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr"/>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>עורך דין ניהול עזבון בביתר עילית מומלץ</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>info@lawreviews.co.il</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>https://www.lawreviews.co.il/search/service/estate-management/jerusalem/betar-illit</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>09673393</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr"/>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>ניהול נכסים באלעד</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>callibenatar@gmail.com</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>https://perfecto-holdings.co.il/asset-management-elad/</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>0250120</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>ארקל ניהול ואחזקת מבנים</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>arkal.clean@gmail.com</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>https://ar-kal.co.il/</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>033818100</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr"/>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>ניהול ואחזקת מבנים: ראשי - הכל TOP בע״מ</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>office.alltop@gmail.com</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>https://alltop.co.il/</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>0509144434</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr"/>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>אודות</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>office@meitav-manage.co.il</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>https://meitav-manage.co.il/%D7%90%D7%95%D7%93%D7%95%D7%AA/</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>0240708</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr"/>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>רשת מתנ"סים שפרעם (ע"ר) | עמותה</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>site3@justice.force.com</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>https://www.guidestar.org.il/he/organization/580629954</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>0557668262</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr"/>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>קידוחי סחנין בע"מ</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>support@conwize.co.il</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>https://conwize.co.il/directory/companies/84622459fc58eb2f82a7?lang=he</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>0401851343</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr"/>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>ב.ליטאי אר.או.אל - ניהול סיכונים בע"מ</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>b-litay@litay-rim.co.il</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>https://litay-rim.co.il/</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>0260528</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr"/>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>מכלול הנדסה: עמוד הבית</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>office@mihlol.co.il</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>https://mihlol.co.il/</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>0230823</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr"/>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>חכל אופקים: בית</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>לoffice@hcl.co.il</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>https://hcl-ofaqim.co.il/</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>0221211</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr"/>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>שירותי המינהלת - אזורי התעשייה אופקים</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>u00a0ilanh@hcl.co.il</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>https://ofaqimindustry.co.il/%D7%A9%D7%99%D7%A8%D7%95%D7%AA%D7%99-%D7%94%D7%9E%D7%99%D7%A0%D7%94%D7%9C%D7%AA/</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>0190822</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr"/>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>יהלום ניהול ואחזקה – ניהול ואחזקת בתים משותפים ומשרדים</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>nihul.yahalom@gmail.com</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>https://nihul-yahalom.co.il/</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>0773626400</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 15 new companies 2026-07-17
</commit_message>
<xml_diff>
--- a/master_companies.xlsx
+++ b/master_companies.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:I77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1661,10 +1661,8 @@
           <t>https://www.bhomeisr.co.il/%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%A0%D7%9B%D7%A1%D7%99%D7%9D-%D7%91%D7%99%D7%A8%D7%95%D7%A9%D7%9C%D7%99%D7%9D/</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>0260601</t>
-        </is>
+      <c r="F38" t="n">
+        <v>260601</v>
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
@@ -1688,10 +1686,8 @@
           <t>https://www.natoon-group.co.il/</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>0946182035</t>
-        </is>
+      <c r="F39" t="n">
+        <v>946182035</v>
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr"/>
@@ -1715,10 +1711,8 @@
           <t>https://www.paxnihul.co.il/</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>0547755722</t>
-        </is>
+      <c r="F40" t="n">
+        <v>547755722</v>
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr"/>
@@ -1746,10 +1740,8 @@
           <t>https://belms.co.il/</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>0547654078</t>
-        </is>
+      <c r="F41" t="n">
+        <v>547654078</v>
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
@@ -1773,10 +1765,8 @@
           <t>https://kgat.co.il/</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>0260209</t>
-        </is>
+      <c r="F42" t="n">
+        <v>260209</v>
       </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr"/>
@@ -1800,10 +1790,8 @@
           <t>https://www.ysgat.co.il/</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>0230420</t>
-        </is>
+      <c r="F43" t="n">
+        <v>230420</v>
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
@@ -1827,10 +1815,8 @@
           <t>https://www.enosh.org.il/%D7%9E%D7%A8%D7%9B%D7%96%D7%99%D7%9D/%D7%90%D7%95%D7%9D-%D7%90%D7%9C-%D7%A4%D7%97%D7%9D/</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>0250609</t>
-        </is>
+      <c r="F44" t="n">
+        <v>250609</v>
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr"/>
@@ -1854,10 +1840,8 @@
           <t>https://www.sba.org.il/hb/MaofServices/courses/Pages/Um_El_Fahem/gen-27-10-21.aspx</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>0771233176</t>
-        </is>
+      <c r="F45" t="n">
+        <v>771233176</v>
       </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr"/>
@@ -1881,10 +1865,8 @@
           <t>https://icomplex.co.il/</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>0777060504</t>
-        </is>
+      <c r="F46" t="n">
+        <v>777060504</v>
       </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr"/>
@@ -1908,10 +1890,8 @@
           <t>https://www.all-service.co.il/</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>0220222</t>
-        </is>
+      <c r="F47" t="n">
+        <v>220222</v>
       </c>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr"/>
@@ -1935,10 +1915,8 @@
           <t>https://calliber.co.il/building-maintenance-maale-adumim/</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>043417951853</t>
-        </is>
+      <c r="F48" t="n">
+        <v>43417951853</v>
       </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr"/>
@@ -1962,10 +1940,8 @@
           <t>https://www.tarbut-hadiur.gov.il/content/142</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>0733485610</t>
-        </is>
+      <c r="F49" t="n">
+        <v>733485610</v>
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
@@ -1989,10 +1965,8 @@
           <t>https://perfecto-holdings.co.il/building-cleaning-maale-adumim/</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>0250120</t>
-        </is>
+      <c r="F50" t="n">
+        <v>250120</v>
       </c>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr"/>
@@ -2016,10 +1990,8 @@
           <t>https://www.lawreviews.co.il/search/service/estate-management/jerusalem/betar-illit</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>09673393</t>
-        </is>
+      <c r="F51" t="n">
+        <v>9673393</v>
       </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr"/>
@@ -2043,10 +2015,8 @@
           <t>https://perfecto-holdings.co.il/asset-management-elad/</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>0250120</t>
-        </is>
+      <c r="F52" t="n">
+        <v>250120</v>
       </c>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr"/>
@@ -2070,10 +2040,8 @@
           <t>https://ar-kal.co.il/</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>033818100</t>
-        </is>
+      <c r="F53" t="n">
+        <v>33818100</v>
       </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr"/>
@@ -2097,10 +2065,8 @@
           <t>https://alltop.co.il/</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>0509144434</t>
-        </is>
+      <c r="F54" t="n">
+        <v>509144434</v>
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr"/>
@@ -2124,10 +2090,8 @@
           <t>https://meitav-manage.co.il/%D7%90%D7%95%D7%93%D7%95%D7%AA/</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>0240708</t>
-        </is>
+      <c r="F55" t="n">
+        <v>240708</v>
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr"/>
@@ -2151,10 +2115,8 @@
           <t>https://www.guidestar.org.il/he/organization/580629954</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>0557668262</t>
-        </is>
+      <c r="F56" t="n">
+        <v>557668262</v>
       </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr"/>
@@ -2178,10 +2140,8 @@
           <t>https://conwize.co.il/directory/companies/84622459fc58eb2f82a7?lang=he</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>0401851343</t>
-        </is>
+      <c r="F57" t="n">
+        <v>401851343</v>
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr"/>
@@ -2205,10 +2165,8 @@
           <t>https://litay-rim.co.il/</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>0260528</t>
-        </is>
+      <c r="F58" t="n">
+        <v>260528</v>
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr"/>
@@ -2232,10 +2190,8 @@
           <t>https://mihlol.co.il/</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>0230823</t>
-        </is>
+      <c r="F59" t="n">
+        <v>230823</v>
       </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr"/>
@@ -2259,10 +2215,8 @@
           <t>https://hcl-ofaqim.co.il/</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>0221211</t>
-        </is>
+      <c r="F60" t="n">
+        <v>221211</v>
       </c>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr"/>
@@ -2286,10 +2240,8 @@
           <t>https://ofaqimindustry.co.il/%D7%A9%D7%99%D7%A8%D7%95%D7%AA%D7%99-%D7%94%D7%9E%D7%99%D7%A0%D7%94%D7%9C%D7%AA/</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>0190822</t>
-        </is>
+      <c r="F61" t="n">
+        <v>190822</v>
       </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr"/>
@@ -2313,14 +2265,449 @@
           <t>https://nihul-yahalom.co.il/</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>0773626400</t>
-        </is>
+      <c r="F62" t="n">
+        <v>773626400</v>
       </c>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr"/>
       <c r="I62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr"/>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>פרויקטים - חברת יקיר בע"מ</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>בני ברק</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>itay@yakirb.co.il</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>https://yakirb.co.il/%D7%A4%D7%A8%D7%95%D7%99%D7%A7%D7%98%D7%99%D7%9D/</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>0220502</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr"/>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>ניהול ב.ס.ר. 4 בע"מ - 515524171 - CheckID</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>בני ברק</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>irena@yakirb.co.il</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>https://www.checkid.co.il/company/%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%91.%D7%A1.%D7%A8.-4-%D7%91%D7%A2~%D7%9E-515524171</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>036819558</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr"/>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>ניהול נכסים בבני ברק</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>בני ברק</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>documentsite@gmail.com</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>https://renthouse.co.il/%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%A0%D7%9B%D7%A1%D7%99%D7%9D-%D7%91%D7%91%D7%A0%D7%99-%D7%91%D7%A8%D7%A7/</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>0250107</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr"/>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>ניהול ואחזקת מבנים בחולון | ניהול ועד בית בחולון</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>חולון</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>roi@mvm.co.il</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>https://www.t-grp.co.il/%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%95%D7%90%D7%97%D7%96%D7%A7%D7%AA-%D7%9E%D7%91%D7%A0%D7%99%D7%9D-%D7%91%D7%97%D7%95%D7%9C%D7%95%D7%9F</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>031324060739</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr"/>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>ניהול AirBnb ודירות נופש באילת​ - EasyBnb Israel</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>אילת</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>info@easybnb.co.il</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>https://easybnb.co.il/</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>0231225</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr"/>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>ניהול מבנים באשקלון, אחזקת מבנים באשקלון, יוסף אחזקות</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>אשקלון</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>yoseffix@gmail.com</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>https://www.asakim.co.il/yosefix/</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>005202015231</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr"/>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>מעיין גנים ניהול ואחזקת מבנים: דף הבית</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Office@m-ganim.co.il</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>https://maayan-ganim.co.il/</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>0260601</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr"/>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>ניהול נכסים בקרית שמונה - נדל"ן מבוסס נתונים - Bashiri - תיווך קרית ...</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>office@bashiri.co.il</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>https://bashiri.co.il/%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%A0%D7%9B%D7%A1%D7%99%D7%9D/</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>0230216</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr"/>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>ניקיון עכו - neptun</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>info@neptun.co.il</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>https://neptun.co.il/acre-cleaning/</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>0220911</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr"/>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>אודות - moreng.co.il</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>mor_office@moreng.co.il</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>https://moreng.co.il/%D7%90%D7%95%D7%93%D7%95%D7%AA/</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>026283098</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr"/>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>א.ד. רהט הנדסה - מִנהלת פארק היי טק הר-חוצבים</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>ירושלים</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>office@e-rahat.co.il</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>https://hotzvim.org.il/company/%D7%90-%D7%93-%D7%A8%D7%94%D7%98-%D7%94%D7%A0%D7%93%D7%A1%D7%94/</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>025870071</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr"/>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>אחזקת מבנים במגדל העמק - טופ קלין שירות מקצועי ואמין</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr"/>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>jgtopclean@gmail.com</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>https://jgtopclean.co.il/building-maintenance-migdal-haemek/</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>0251018</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr"/>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>ניהול פרויקטים הנדסיים, חברת ניהול פרויקטים - in-project: אין פרוגקט</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr"/>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>office1@inproject.co.il</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>https://www.in-project.co.il/</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>0251203</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr"/>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>MSP | ניהול בתים משותפים</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>תל אביב</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>msptlv@gmail.com</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>https://www.msp.org.il/</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>0250527</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr"/>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>"בית בטוח" - חברת בוטיק לניהול ועדי בתים, ניהול בתים משותפים ונכסים ...</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr"/>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>safehouse777@gmail.com</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>https://www.safehouse.org.il/</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>0775549921</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr"/>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 11 new companies 2026-07-24
</commit_message>
<xml_diff>
--- a/master_companies.xlsx
+++ b/master_companies.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I77"/>
+  <dimension ref="A1:I88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2294,10 +2294,8 @@
           <t>https://yakirb.co.il/%D7%A4%D7%A8%D7%95%D7%99%D7%A7%D7%98%D7%99%D7%9D/</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>0220502</t>
-        </is>
+      <c r="F63" t="n">
+        <v>220502</v>
       </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr"/>
@@ -2325,10 +2323,8 @@
           <t>https://www.checkid.co.il/company/%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%91.%D7%A1.%D7%A8.-4-%D7%91%D7%A2~%D7%9E-515524171</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>036819558</t>
-        </is>
+      <c r="F64" t="n">
+        <v>36819558</v>
       </c>
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr"/>
@@ -2356,10 +2352,8 @@
           <t>https://renthouse.co.il/%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%A0%D7%9B%D7%A1%D7%99%D7%9D-%D7%91%D7%91%D7%A0%D7%99-%D7%91%D7%A8%D7%A7/</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>0250107</t>
-        </is>
+      <c r="F65" t="n">
+        <v>250107</v>
       </c>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr"/>
@@ -2387,10 +2381,8 @@
           <t>https://www.t-grp.co.il/%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%95%D7%90%D7%97%D7%96%D7%A7%D7%AA-%D7%9E%D7%91%D7%A0%D7%99%D7%9D-%D7%91%D7%97%D7%95%D7%9C%D7%95%D7%9F</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>031324060739</t>
-        </is>
+      <c r="F66" t="n">
+        <v>31324060739</v>
       </c>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr"/>
@@ -2418,10 +2410,8 @@
           <t>https://easybnb.co.il/</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>0231225</t>
-        </is>
+      <c r="F67" t="n">
+        <v>231225</v>
       </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr"/>
@@ -2449,10 +2439,8 @@
           <t>https://www.asakim.co.il/yosefix/</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>005202015231</t>
-        </is>
+      <c r="F68" t="n">
+        <v>5202015231</v>
       </c>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr"/>
@@ -2476,10 +2464,8 @@
           <t>https://maayan-ganim.co.il/</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>0260601</t>
-        </is>
+      <c r="F69" t="n">
+        <v>260601</v>
       </c>
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr"/>
@@ -2503,10 +2489,8 @@
           <t>https://bashiri.co.il/%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%A0%D7%9B%D7%A1%D7%99%D7%9D/</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>0230216</t>
-        </is>
+      <c r="F70" t="n">
+        <v>230216</v>
       </c>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr"/>
@@ -2530,10 +2514,8 @@
           <t>https://neptun.co.il/acre-cleaning/</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>0220911</t>
-        </is>
+      <c r="F71" t="n">
+        <v>220911</v>
       </c>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr"/>
@@ -2557,10 +2539,8 @@
           <t>https://moreng.co.il/%D7%90%D7%95%D7%93%D7%95%D7%AA/</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>026283098</t>
-        </is>
+      <c r="F72" t="n">
+        <v>26283098</v>
       </c>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr"/>
@@ -2588,10 +2568,8 @@
           <t>https://hotzvim.org.il/company/%D7%90-%D7%93-%D7%A8%D7%94%D7%98-%D7%94%D7%A0%D7%93%D7%A1%D7%94/</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>025870071</t>
-        </is>
+      <c r="F73" t="n">
+        <v>25870071</v>
       </c>
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr"/>
@@ -2615,10 +2593,8 @@
           <t>https://jgtopclean.co.il/building-maintenance-migdal-haemek/</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>0251018</t>
-        </is>
+      <c r="F74" t="n">
+        <v>251018</v>
       </c>
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr"/>
@@ -2642,10 +2618,8 @@
           <t>https://www.in-project.co.il/</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>0251203</t>
-        </is>
+      <c r="F75" t="n">
+        <v>251203</v>
       </c>
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr"/>
@@ -2673,10 +2647,8 @@
           <t>https://www.msp.org.il/</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>0250527</t>
-        </is>
+      <c r="F76" t="n">
+        <v>250527</v>
       </c>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr"/>
@@ -2700,14 +2672,325 @@
           <t>https://www.safehouse.org.il/</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>0775549921</t>
-        </is>
+      <c r="F77" t="n">
+        <v>775549921</v>
       </c>
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr"/>
       <c r="I77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr"/>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>שרמן ניהול ואחזקות מבנים — ניהול מבנים מוביל בתל אביב</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>תל אביב</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>info@sherman-group.co.il</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>https://www.sherman-group.co.il/</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>0583837777</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr"/>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>שירותי תחזוקת מבנים וניקיון</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>באר שבע</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>office@capi-tal.co.il</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>https://www.capi-tal.co.il/</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>0260701</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr"/>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>שיא הברכה – ניהול ואחזקת מבנים</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr"/>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>office@si-b.co.il</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>https://si-b.co.il/</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>0522863889</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr"/>
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr"/>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>קריית שמונה</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr"/>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>office@maavarimg.org.il</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>https://taasuka.galil-elion.org.il/he/%D7%9E%D7%95%D7%A2%D7%A6%D7%94%D7%90%D7%96%D7%95%D7%A8/%D7%A7%D7%A8%D7%99%D7%99%D7%AA-%D7%A9%D7%9E%D7%95%D7%A0%D7%94</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>0260724</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr"/>
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr"/>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>אאורה קריית ביאליק - התחדשות עירונית קרית ביאליק</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr"/>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>orit.s@auraisrael.co.il</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>https://auraisrael.co.il/project/%D7%90%D7%90%D7%95%D7%A8%D7%94-%D7%A7%D7%A8%D7%99%D7%99%D7%AA-%D7%91%D7%99%D7%90%D7%9C%D7%99%D7%A7/</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>0251201</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr"/>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>5 כוכבים – תנו לנו לדאוג לבניין שלכם כדי שאתם תהיו בראש שקט</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr"/>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>sb.five.stars@gmail.com</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>https://www.five-stars.co.il/</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>0528895498</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr"/>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>חברת תגל | ניהול | הנדסה אזרחית - טירת בכרמל / ת"א</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>רמת גן</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>office@tagal.co.il</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>https://www.tagal.co.il/</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>02320233</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr"/>
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr"/>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Kendu – הופכים רעיונות יצירתיים למוצרים מצליחים</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>הרצליה</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>adielshfaram@gmail.com</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>https://kendu.co.il/</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>042179217</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr"/>
+      <c r="H85" t="inlineStr"/>
+      <c r="I85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr"/>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>קבוצת גדיש: Home</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr"/>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>info@gadish.co.il</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>https://www.gadish.co.il/</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>03070308</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr"/>
+      <c r="H86" t="inlineStr"/>
+      <c r="I86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr"/>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>ירוחם</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr"/>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>info@ranwolf.co.il</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>https://www.ranwolf.co.il/yerucham</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>00175568691</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr"/>
+      <c r="H87" t="inlineStr"/>
+      <c r="I87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr"/>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>תוכנה לניהול אחזקת מבנים- כל המושגים שכדאי להכיר בתחום ...</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr"/>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>top-privacy@top-group.co.il</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>https://www.ramdor.co.il/articles/maintaining-buildings-is-important-concepts/</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>0190922</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr"/>
+      <c r="H88" t="inlineStr"/>
+      <c r="I88" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 8 new companies 2026-08-14
</commit_message>
<xml_diff>
--- a/master_companies.xlsx
+++ b/master_companies.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I88"/>
+  <dimension ref="A1:I96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2701,10 +2701,8 @@
           <t>https://www.sherman-group.co.il/</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>0583837777</t>
-        </is>
+      <c r="F78" t="n">
+        <v>583837777</v>
       </c>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr"/>
@@ -2732,10 +2730,8 @@
           <t>https://www.capi-tal.co.il/</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>0260701</t>
-        </is>
+      <c r="F79" t="n">
+        <v>260701</v>
       </c>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr"/>
@@ -2759,10 +2755,8 @@
           <t>https://si-b.co.il/</t>
         </is>
       </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>0522863889</t>
-        </is>
+      <c r="F80" t="n">
+        <v>522863889</v>
       </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr"/>
@@ -2786,10 +2780,8 @@
           <t>https://taasuka.galil-elion.org.il/he/%D7%9E%D7%95%D7%A2%D7%A6%D7%94%D7%90%D7%96%D7%95%D7%A8/%D7%A7%D7%A8%D7%99%D7%99%D7%AA-%D7%A9%D7%9E%D7%95%D7%A0%D7%94</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>0260724</t>
-        </is>
+      <c r="F81" t="n">
+        <v>260724</v>
       </c>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr"/>
@@ -2813,10 +2805,8 @@
           <t>https://auraisrael.co.il/project/%D7%90%D7%90%D7%95%D7%A8%D7%94-%D7%A7%D7%A8%D7%99%D7%99%D7%AA-%D7%91%D7%99%D7%90%D7%9C%D7%99%D7%A7/</t>
         </is>
       </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>0251201</t>
-        </is>
+      <c r="F82" t="n">
+        <v>251201</v>
       </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr"/>
@@ -2840,10 +2830,8 @@
           <t>https://www.five-stars.co.il/</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>0528895498</t>
-        </is>
+      <c r="F83" t="n">
+        <v>528895498</v>
       </c>
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr"/>
@@ -2871,10 +2859,8 @@
           <t>https://www.tagal.co.il/</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t>02320233</t>
-        </is>
+      <c r="F84" t="n">
+        <v>2320233</v>
       </c>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr"/>
@@ -2902,10 +2888,8 @@
           <t>https://kendu.co.il/</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>042179217</t>
-        </is>
+      <c r="F85" t="n">
+        <v>42179217</v>
       </c>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr"/>
@@ -2929,10 +2913,8 @@
           <t>https://www.gadish.co.il/</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>03070308</t>
-        </is>
+      <c r="F86" t="n">
+        <v>3070308</v>
       </c>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr"/>
@@ -2956,10 +2938,8 @@
           <t>https://www.ranwolf.co.il/yerucham</t>
         </is>
       </c>
-      <c r="F87" t="inlineStr">
-        <is>
-          <t>00175568691</t>
-        </is>
+      <c r="F87" t="n">
+        <v>175568691</v>
       </c>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr"/>
@@ -2983,14 +2963,232 @@
           <t>https://www.ramdor.co.il/articles/maintaining-buildings-is-important-concepts/</t>
         </is>
       </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>0190922</t>
-        </is>
+      <c r="F88" t="n">
+        <v>190922</v>
       </c>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr"/>
       <c r="I88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr"/>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>bgholdings: B.G. Holdings - home 180520</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>נתניה</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>info@website.com</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>https://bgmanage.co.il/</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>0542454345</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr"/>
+      <c r="H89" t="inlineStr"/>
+      <c r="I89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr"/>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>יארה אחזקות: בית</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr"/>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>office@yara-h.co.il</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>https://yara-h.co.il/</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>0251119</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr"/>
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr"/>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>ניהול בתים משותפים בגבעתיים | האוס אפ - House-Up</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr"/>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Abm1dao@gmail.com</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>https://house-up.co.il/%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%91%D7%AA%D7%99%D7%9D-%D7%9E%D7%A9%D7%95%D7%AA%D7%A4%D7%99%D7%9D-%D7%91%D7%92%D7%91%D7%A2%D7%AA%D7%99%D7%99%D7%9D/</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>0260314</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr"/>
+      <c r="H91" t="inlineStr"/>
+      <c r="I91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr"/>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>A.G.R ניהול מבנים ואחזקה. כוח אדם בעמ</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr"/>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>agrnofar@gmail.com</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>https://nadlano.co.il/office/management-21502/</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>042820017</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr"/>
+      <c r="H92" t="inlineStr"/>
+      <c r="I92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr"/>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>שירותי ניקיון לבניינים | שחר מור - ניהול ואחזקת מבנים | Rehovot</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr"/>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>elad@shaharmor.co.il</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>https://www.shaharmor.co.il/</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>089454954</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr"/>
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr"/>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>ג.ש.ר (נדב אורסטי) חברת אחזקה לבניין | ניהול ועד בית</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr"/>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>nbnadav@gmail.com</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>https://nadlano.co.il/office/management-6546/</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>0523914927</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr"/>
+      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr"/>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>המכרזים של החברה הכלכלית לפיתוח ירוחם</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr"/>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>daniel@benin.co.il</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>https://www.michrazim.org.il/authorities/%D7%94%D7%97%D7%91%D7%A8%D7%94-%D7%94%D7%9B%D7%9C%D7%9B%D7%9C%D7%99%D7%AA-%D7%9C%D7%A4%D7%99%D7%AA%D7%95%D7%97-%D7%99%D7%A8%D7%95%D7%97%D7%9D</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>00663145</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr"/>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr"/>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>נכסי אריאל: חברת ניהול נכסים ומבנים המובילה בישראל</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr"/>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>shanish@electra.co.il</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>https://www.arielgroup.co.il/</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>011550282</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr"/>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 1 new companies 2026-08-21
</commit_message>
<xml_diff>
--- a/master_companies.xlsx
+++ b/master_companies.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I96"/>
+  <dimension ref="A1:I97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2992,10 +2992,8 @@
           <t>https://bgmanage.co.il/</t>
         </is>
       </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>0542454345</t>
-        </is>
+      <c r="F89" t="n">
+        <v>542454345</v>
       </c>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr"/>
@@ -3019,10 +3017,8 @@
           <t>https://yara-h.co.il/</t>
         </is>
       </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>0251119</t>
-        </is>
+      <c r="F90" t="n">
+        <v>251119</v>
       </c>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr"/>
@@ -3046,10 +3042,8 @@
           <t>https://house-up.co.il/%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%91%D7%AA%D7%99%D7%9D-%D7%9E%D7%A9%D7%95%D7%AA%D7%A4%D7%99%D7%9D-%D7%91%D7%92%D7%91%D7%A2%D7%AA%D7%99%D7%99%D7%9D/</t>
         </is>
       </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>0260314</t>
-        </is>
+      <c r="F91" t="n">
+        <v>260314</v>
       </c>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr"/>
@@ -3073,10 +3067,8 @@
           <t>https://nadlano.co.il/office/management-21502/</t>
         </is>
       </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>042820017</t>
-        </is>
+      <c r="F92" t="n">
+        <v>42820017</v>
       </c>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr"/>
@@ -3100,10 +3092,8 @@
           <t>https://www.shaharmor.co.il/</t>
         </is>
       </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>089454954</t>
-        </is>
+      <c r="F93" t="n">
+        <v>89454954</v>
       </c>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr"/>
@@ -3127,10 +3117,8 @@
           <t>https://nadlano.co.il/office/management-6546/</t>
         </is>
       </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>0523914927</t>
-        </is>
+      <c r="F94" t="n">
+        <v>523914927</v>
       </c>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr"/>
@@ -3154,10 +3142,8 @@
           <t>https://www.michrazim.org.il/authorities/%D7%94%D7%97%D7%91%D7%A8%D7%94-%D7%94%D7%9B%D7%9C%D7%9B%D7%9C%D7%99%D7%AA-%D7%9C%D7%A4%D7%99%D7%AA%D7%95%D7%97-%D7%99%D7%A8%D7%95%D7%97%D7%9D</t>
         </is>
       </c>
-      <c r="F95" t="inlineStr">
-        <is>
-          <t>00663145</t>
-        </is>
+      <c r="F95" t="n">
+        <v>663145</v>
       </c>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr"/>
@@ -3181,14 +3167,43 @@
           <t>https://www.arielgroup.co.il/</t>
         </is>
       </c>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>011550282</t>
-        </is>
+      <c r="F96" t="n">
+        <v>11550282</v>
       </c>
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr"/>
       <c r="I96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr"/>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>הנדסה אזרחית (בניין) - ניהול + תכנון - كلية الهندسيين سخنين</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>רחובות</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>sac.org.il@gmail.com</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>https://sac.org.il/he/%D7%94%D7%A0%D7%93%D7%A1%D7%94-%D7%90%D7%96%D7%A8%D7%97%D7%99%D7%AA-%D7%94%D7%A0%D7%93%D7%A1%D7%AA-%D7%91%D7%A0%D7%99%D7%99%D7%9F-%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%AA%D7%9B%D7%A0%D7%95%D7%9F/</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>0260707</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr"/>
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 4 new companies 2026-08-28
</commit_message>
<xml_diff>
--- a/master_companies.xlsx
+++ b/master_companies.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I97"/>
+  <dimension ref="A1:I101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3196,14 +3196,120 @@
           <t>https://sac.org.il/he/%D7%94%D7%A0%D7%93%D7%A1%D7%94-%D7%90%D7%96%D7%A8%D7%97%D7%99%D7%AA-%D7%94%D7%A0%D7%93%D7%A1%D7%AA-%D7%91%D7%A0%D7%99%D7%99%D7%9F-%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%AA%D7%9B%D7%A0%D7%95%D7%9F/</t>
         </is>
       </c>
-      <c r="F97" t="inlineStr">
-        <is>
-          <t>0260707</t>
-        </is>
+      <c r="F97" t="n">
+        <v>260707</v>
       </c>
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="inlineStr"/>
       <c r="I97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr"/>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>נירו ניהול ואחזקת מבנים</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr"/>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>niro@tigboret.co.il</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>https://niro360.co.il/</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>0260409</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr"/>
+      <c r="H98" t="inlineStr"/>
+      <c r="I98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr"/>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>אור ניהול ואחזקת מבנים</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr"/>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Erez@ornihul.com</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>https://greenbook.co.il/card/7644/19000</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>0503977046</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr"/>
+      <c r="H99" t="inlineStr"/>
+      <c r="I99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr"/>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>אדן אור ניהול ואחזקות מבנים בע"מ: תחזוקת מבנים</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr"/>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>eden.manag@walla.com</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>https://eden-or.zapweb.co.il/</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>0737533575</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr"/>
+      <c r="H100" t="inlineStr"/>
+      <c r="I100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr"/>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>מכרז פומבי 16/25: מכרז מסגרת לקבלת הצעות לשירותי ניהול תכנון ...</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr"/>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>katya@ylc.org.il</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>https://www.calcalit-yeruham.co.il/product/2649</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>089201208</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr"/>
+      <c r="H101" t="inlineStr"/>
+      <c r="I101" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>